<commit_message>
devi week 6 material & timesheet
</commit_message>
<xml_diff>
--- a/DeviMaya_S388017/Timesheet Devi Maya.xlsx
+++ b/DeviMaya_S388017/Timesheet Devi Maya.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/devi/Documents/GitHub/PRT585-SOFTWARE-ENGINEERING-PRACTICE/DeviMaya_S388017/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3142B6D-A640-A949-BBFD-FF40AF0926AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2D952FD-538C-5148-B010-923029E661B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Individual timesheet" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="53">
   <si>
     <t>EACH INDIVIDUAL MUST HAVE TO ENTER 6 HOURS TIME LOGGING IN THIS PAGE PER EACH WEEK</t>
   </si>
@@ -185,13 +185,34 @@
   </si>
   <si>
     <t>Individual study: SecureVault (finish 1E)</t>
+  </si>
+  <si>
+    <t>Prepare BA &amp; DA study pathway document</t>
+  </si>
+  <si>
+    <t>Finish activity diagram</t>
+  </si>
+  <si>
+    <t>Week-6</t>
+  </si>
+  <si>
+    <t>BA: self-study system design, dropbox case study</t>
+  </si>
+  <si>
+    <t>BA: self-study system design, dropbox case study (finish domain-related FR and NFR)</t>
+  </si>
+  <si>
+    <t>DA: self-study system design, dropbox case study</t>
+  </si>
+  <si>
+    <t>DA: self-study system design, dropbox case study (finish conceptual entity list, capacity estimation practice)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -265,14 +286,6 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -396,20 +409,20 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -950,7 +963,7 @@
       <c r="D14" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="24" t="s">
         <v>23</v>
       </c>
     </row>
@@ -967,7 +980,7 @@
       <c r="D15" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="24" t="s">
         <v>24</v>
       </c>
     </row>
@@ -975,7 +988,7 @@
       <c r="A16"/>
       <c r="B16"/>
       <c r="C16"/>
-      <c r="E16" s="25"/>
+      <c r="E16" s="24"/>
     </row>
     <row r="17" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
@@ -1079,6 +1092,108 @@
         <v>45</v>
       </c>
     </row>
+    <row r="24" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" t="s">
+        <v>8</v>
+      </c>
+      <c r="D24" s="4">
+        <v>1</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25" t="s">
+        <v>8</v>
+      </c>
+      <c r="D25" s="4">
+        <v>2</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" t="s">
+        <v>8</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A27" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B27" t="s">
+        <v>7</v>
+      </c>
+      <c r="C27" t="s">
+        <v>8</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A28" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B28" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" t="s">
+        <v>8</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A29" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" t="s">
+        <v>8</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
     <row r="37" spans="5:5" x14ac:dyDescent="0.2">
       <c r="E37"/>
     </row>
@@ -1095,22 +1210,22 @@
       <c r="E41"/>
     </row>
     <row r="42" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E42" s="24"/>
+      <c r="E42" s="23"/>
     </row>
     <row r="43" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E43" s="24"/>
+      <c r="E43" s="23"/>
     </row>
     <row r="44" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E44" s="24"/>
+      <c r="E44" s="23"/>
     </row>
     <row r="45" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E45" s="24"/>
+      <c r="E45" s="23"/>
     </row>
     <row r="46" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E46" s="24"/>
+      <c r="E46" s="23"/>
     </row>
     <row r="47" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E47" s="24"/>
+      <c r="E47" s="23"/>
     </row>
     <row r="49" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E49" s="9"/>
@@ -1325,42 +1440,42 @@
       <c r="A130" s="13"/>
       <c r="B130" s="16"/>
       <c r="C130" s="16"/>
-      <c r="D130" s="23"/>
+      <c r="D130" s="22"/>
       <c r="E130" s="17"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" s="13"/>
       <c r="B131" s="16"/>
       <c r="C131" s="16"/>
-      <c r="D131" s="23"/>
+      <c r="D131" s="22"/>
       <c r="E131" s="17"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" s="13"/>
       <c r="B132" s="16"/>
       <c r="C132" s="16"/>
-      <c r="D132" s="23"/>
+      <c r="D132" s="22"/>
       <c r="E132" s="16"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" s="13"/>
       <c r="B133" s="16"/>
       <c r="C133" s="16"/>
-      <c r="D133" s="23"/>
+      <c r="D133" s="22"/>
       <c r="E133" s="17"/>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" s="13"/>
       <c r="B134" s="16"/>
       <c r="C134" s="16"/>
-      <c r="D134" s="23"/>
+      <c r="D134" s="22"/>
       <c r="E134" s="17"/>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135" s="13"/>
       <c r="B135" s="16"/>
       <c r="C135" s="16"/>
-      <c r="D135" s="23"/>
+      <c r="D135" s="22"/>
       <c r="E135" s="17"/>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.2">
@@ -1384,56 +1499,56 @@
     <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144" s="13"/>
       <c r="B144" s="16"/>
-      <c r="E144" s="21"/>
+      <c r="E144" s="20"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145" s="13"/>
       <c r="B145" s="16"/>
-      <c r="E145" s="21"/>
+      <c r="E145" s="20"/>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146" s="13"/>
       <c r="B146" s="16"/>
-      <c r="E146" s="21"/>
+      <c r="E146" s="20"/>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147" s="13"/>
       <c r="B147" s="16"/>
-      <c r="E147" s="22"/>
+      <c r="E147" s="21"/>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" s="13"/>
       <c r="B148" s="16"/>
-      <c r="E148" s="21"/>
+      <c r="E148" s="20"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149" s="13"/>
       <c r="B149" s="16"/>
-      <c r="E149" s="21"/>
+      <c r="E149" s="20"/>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" s="13"/>
-      <c r="B151" s="20"/>
+      <c r="B151" s="19"/>
       <c r="E151" s="17"/>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" s="13"/>
-      <c r="B152" s="20"/>
+      <c r="B152" s="19"/>
       <c r="E152" s="17"/>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" s="13"/>
-      <c r="B153" s="20"/>
+      <c r="B153" s="19"/>
       <c r="E153" s="16"/>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" s="13"/>
-      <c r="B154" s="20"/>
+      <c r="B154" s="19"/>
       <c r="E154" s="17"/>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" s="13"/>
-      <c r="B155" s="20"/>
+      <c r="B155" s="19"/>
       <c r="E155" s="17"/>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.2">
@@ -1493,17 +1608,17 @@
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A175" s="13"/>
-      <c r="B175" s="20"/>
+      <c r="B175" s="19"/>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A176" s="13"/>
-      <c r="B176" s="20"/>
+      <c r="B176" s="19"/>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A177" s="13"/>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A178" s="20"/>
+      <c r="A178" s="19"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
@@ -1744,7 +1859,7 @@
       <c r="D15" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="24" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1765,28 +1880,79 @@
         <v>39</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B17"/>
       <c r="C17"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B18"/>
-      <c r="C18"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B19"/>
-      <c r="C19"/>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B20"/>
-      <c r="C20"/>
-      <c r="E20" s="19"/>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B21"/>
-      <c r="C21"/>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" s="25" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" s="25" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B22"/>
       <c r="C22"/>
     </row>
@@ -1806,22 +1972,22 @@
       <c r="E41"/>
     </row>
     <row r="42" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E42" s="24"/>
+      <c r="E42" s="23"/>
     </row>
     <row r="43" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E43" s="24"/>
+      <c r="E43" s="23"/>
     </row>
     <row r="44" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E44" s="24"/>
+      <c r="E44" s="23"/>
     </row>
     <row r="45" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E45" s="24"/>
+      <c r="E45" s="23"/>
     </row>
     <row r="46" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E46" s="24"/>
+      <c r="E46" s="23"/>
     </row>
     <row r="47" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E47" s="24"/>
+      <c r="E47" s="23"/>
     </row>
     <row r="49" spans="4:5" x14ac:dyDescent="0.2">
       <c r="E49" s="9"/>
@@ -2036,42 +2202,42 @@
       <c r="A130" s="13"/>
       <c r="B130" s="16"/>
       <c r="C130" s="16"/>
-      <c r="D130" s="23"/>
+      <c r="D130" s="22"/>
       <c r="E130" s="17"/>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A131" s="13"/>
       <c r="B131" s="16"/>
       <c r="C131" s="16"/>
-      <c r="D131" s="23"/>
+      <c r="D131" s="22"/>
       <c r="E131" s="17"/>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A132" s="13"/>
       <c r="B132" s="16"/>
       <c r="C132" s="16"/>
-      <c r="D132" s="23"/>
+      <c r="D132" s="22"/>
       <c r="E132" s="16"/>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A133" s="13"/>
       <c r="B133" s="16"/>
       <c r="C133" s="16"/>
-      <c r="D133" s="23"/>
+      <c r="D133" s="22"/>
       <c r="E133" s="17"/>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A134" s="13"/>
       <c r="B134" s="16"/>
       <c r="C134" s="16"/>
-      <c r="D134" s="23"/>
+      <c r="D134" s="22"/>
       <c r="E134" s="17"/>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A135" s="13"/>
       <c r="B135" s="16"/>
       <c r="C135" s="16"/>
-      <c r="D135" s="23"/>
+      <c r="D135" s="22"/>
       <c r="E135" s="17"/>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.2">
@@ -2095,56 +2261,56 @@
     <row r="144" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A144" s="13"/>
       <c r="B144" s="16"/>
-      <c r="E144" s="21"/>
+      <c r="E144" s="20"/>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A145" s="13"/>
       <c r="B145" s="16"/>
-      <c r="E145" s="21"/>
+      <c r="E145" s="20"/>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A146" s="13"/>
       <c r="B146" s="16"/>
-      <c r="E146" s="21"/>
+      <c r="E146" s="20"/>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A147" s="13"/>
       <c r="B147" s="16"/>
-      <c r="E147" s="22"/>
+      <c r="E147" s="21"/>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A148" s="13"/>
       <c r="B148" s="16"/>
-      <c r="E148" s="21"/>
+      <c r="E148" s="20"/>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A149" s="13"/>
       <c r="B149" s="16"/>
-      <c r="E149" s="21"/>
+      <c r="E149" s="20"/>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A151" s="13"/>
-      <c r="B151" s="20"/>
+      <c r="B151" s="19"/>
       <c r="E151" s="17"/>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A152" s="13"/>
-      <c r="B152" s="20"/>
+      <c r="B152" s="19"/>
       <c r="E152" s="17"/>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A153" s="13"/>
-      <c r="B153" s="20"/>
+      <c r="B153" s="19"/>
       <c r="E153" s="16"/>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A154" s="13"/>
-      <c r="B154" s="20"/>
+      <c r="B154" s="19"/>
       <c r="E154" s="17"/>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A155" s="13"/>
-      <c r="B155" s="20"/>
+      <c r="B155" s="19"/>
       <c r="E155" s="17"/>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.2">
@@ -2204,17 +2370,17 @@
     </row>
     <row r="175" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A175" s="13"/>
-      <c r="B175" s="20"/>
+      <c r="B175" s="19"/>
     </row>
     <row r="176" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A176" s="13"/>
-      <c r="B176" s="20"/>
+      <c r="B176" s="19"/>
     </row>
     <row r="177" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A177" s="13"/>
     </row>
     <row r="178" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A178" s="20"/>
+      <c r="A178" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>